<commit_message>
Add oracle support to servers
</commit_message>
<xml_diff>
--- a/odcs-template.xlsx
+++ b/odcs-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jochen/Projects/open-data-contract-standard-excel-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58ECC940-E1E1-584B-B311-B4AA053E9340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B8EC82A-F0B9-0B43-8073-AB65EEFA9D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="8" r:id="rId1"/>
@@ -57,25 +57,25 @@
     <definedName name="servers.azure.location">Servers!$C$12</definedName>
     <definedName name="servers.bigquery.dataset">Servers!$C$18</definedName>
     <definedName name="servers.bigquery.project">Servers!$C$17</definedName>
-    <definedName name="servers.custom.account">Servers!$C$62</definedName>
-    <definedName name="servers.custom.catalog">Servers!$C$63</definedName>
-    <definedName name="servers.custom.database">Servers!$C$64</definedName>
-    <definedName name="servers.custom.dataset">Servers!$C$65</definedName>
-    <definedName name="servers.custom.delimiter">Servers!$C$66</definedName>
-    <definedName name="servers.custom.endpointUrl">Servers!$C$67</definedName>
-    <definedName name="servers.custom.format">Servers!$C$68</definedName>
-    <definedName name="servers.custom.host">Servers!$C$69</definedName>
-    <definedName name="servers.custom.location">Servers!$C$70</definedName>
-    <definedName name="servers.custom.path">Servers!$C$71</definedName>
-    <definedName name="servers.custom.port">Servers!$C$72</definedName>
-    <definedName name="servers.custom.project">Servers!$C$73</definedName>
-    <definedName name="servers.custom.region">Servers!$C$74</definedName>
-    <definedName name="servers.custom.regionName">Servers!$C$75</definedName>
-    <definedName name="servers.custom.schema">Servers!$C$76</definedName>
-    <definedName name="servers.custom.serviceName">Servers!$C$77</definedName>
-    <definedName name="servers.custom.stagingDir">Servers!$C$78</definedName>
-    <definedName name="servers.custom.stream">Servers!$C$79</definedName>
-    <definedName name="servers.custom.warehouse">Servers!$C$80</definedName>
+    <definedName name="servers.custom.account">Servers!$C$67</definedName>
+    <definedName name="servers.custom.catalog">Servers!$C$68</definedName>
+    <definedName name="servers.custom.database">Servers!$C$69</definedName>
+    <definedName name="servers.custom.dataset">Servers!$C$70</definedName>
+    <definedName name="servers.custom.delimiter">Servers!$C$71</definedName>
+    <definedName name="servers.custom.endpointUrl">Servers!$C$72</definedName>
+    <definedName name="servers.custom.format">Servers!$C$73</definedName>
+    <definedName name="servers.custom.host">Servers!$C$74</definedName>
+    <definedName name="servers.custom.location">Servers!$C$75</definedName>
+    <definedName name="servers.custom.path">Servers!$C$76</definedName>
+    <definedName name="servers.custom.port">Servers!$C$77</definedName>
+    <definedName name="servers.custom.project">Servers!$C$78</definedName>
+    <definedName name="servers.custom.region">Servers!$C$79</definedName>
+    <definedName name="servers.custom.regionName">Servers!$C$80</definedName>
+    <definedName name="servers.custom.schema">Servers!$C$81</definedName>
+    <definedName name="servers.custom.serviceName">Servers!$C$82</definedName>
+    <definedName name="servers.custom.stagingDir">Servers!$C$83</definedName>
+    <definedName name="servers.custom.stream">Servers!$C$84</definedName>
+    <definedName name="servers.custom.warehouse">Servers!$C$85</definedName>
     <definedName name="servers.databricks.catalog">Servers!$C$21</definedName>
     <definedName name="servers.databricks.host">Servers!$C$23</definedName>
     <definedName name="servers.databricks.schema">Servers!$C$22</definedName>
@@ -87,6 +87,9 @@
     <definedName name="servers.glue.location">Servers!$C$28</definedName>
     <definedName name="servers.kafka.format">Servers!$C$33</definedName>
     <definedName name="servers.kafka.host">Servers!$C$32</definedName>
+    <definedName name="servers.oracle.host">Servers!$C$62</definedName>
+    <definedName name="servers.oracle.port">Servers!$C$63</definedName>
+    <definedName name="servers.oracle.servicename">Servers!$C$64</definedName>
     <definedName name="servers.postgres.database">Servers!$C$38</definedName>
     <definedName name="servers.postgres.host">Servers!$C$36</definedName>
     <definedName name="servers.postgres.port">Servers!$C$37</definedName>
@@ -134,7 +137,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="166">
   <si>
     <t>Property</t>
   </si>
@@ -152,9 +155,6 @@
   </si>
   <si>
     <t>apiVersion</t>
-  </si>
-  <si>
-    <t>v3.0.2</t>
   </si>
   <si>
     <t>Logical Type</t>
@@ -572,9 +572,6 @@
     <t>b)</t>
   </si>
   <si>
-    <t>Open Data Mesh Manager → Go to Data Contracts → Click Add Data Contract → Import from Excel</t>
-  </si>
-  <si>
     <t>Required Properties</t>
   </si>
   <si>
@@ -590,12 +587,6 @@
     <t>datacontract import --format excel --source odcs.xlsx</t>
   </si>
   <si>
-    <t>2025-05-07</t>
-  </si>
-  <si>
-    <t>Or, if you use Data Mesh Manager, import the Excel directly.</t>
-  </si>
-  <si>
     <t>Existing data contracts with the same ID will be updated.</t>
   </si>
   <si>
@@ -633,6 +624,24 @@
   </si>
   <si>
     <t>Comments (internal)</t>
+  </si>
+  <si>
+    <t>2025-12-01</t>
+  </si>
+  <si>
+    <t>Or, if you use Entropy Data, import the Excel directly.</t>
+  </si>
+  <si>
+    <t>Open Entropy Data → Go to Data Contracts → Click Add Data Contract → Import from Excel</t>
+  </si>
+  <si>
+    <t>Oracle</t>
+  </si>
+  <si>
+    <t>ServiceName</t>
+  </si>
+  <si>
+    <t>v3.0.2</t>
   </si>
 </sst>
 </file>
@@ -922,6 +931,21 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -939,21 +963,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1345,7 +1354,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1354,7 +1363,7 @@
     </row>
     <row r="2" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1370,7 +1379,7 @@
     </row>
     <row r="7" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -1383,7 +1392,7 @@
     </row>
     <row r="8" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -1396,7 +1405,7 @@
     </row>
     <row r="9" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
@@ -1409,7 +1418,7 @@
     </row>
     <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -1422,7 +1431,7 @@
     </row>
     <row r="11" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -1457,7 +1466,7 @@
     </row>
     <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
@@ -1470,7 +1479,7 @@
     </row>
     <row r="15" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
@@ -1483,7 +1492,7 @@
     </row>
     <row r="16" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
@@ -1496,7 +1505,7 @@
     </row>
     <row r="17" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
@@ -1509,10 +1518,10 @@
     </row>
     <row r="18" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>140</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>141</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
@@ -1525,7 +1534,7 @@
     <row r="19" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="23"/>
       <c r="B19" s="24" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
@@ -1548,10 +1557,10 @@
     </row>
     <row r="21" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
@@ -1564,7 +1573,7 @@
     <row r="22" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="25"/>
       <c r="B22" s="13" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -1577,7 +1586,7 @@
     <row r="23" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
       <c r="B23" s="13" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
@@ -1611,10 +1620,10 @@
     </row>
     <row r="26" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="13" t="s">
         <v>40</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>41</v>
       </c>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
@@ -1626,10 +1635,10 @@
     </row>
     <row r="27" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
@@ -1641,10 +1650,10 @@
     </row>
     <row r="28" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="13" t="s">
         <v>42</v>
-      </c>
-      <c r="B28" s="13" t="s">
-        <v>43</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
@@ -1705,30 +1714,30 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:2" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B4" s="5"/>
     </row>
     <row r="5" spans="1:2" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B5" s="5"/>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B6" s="5"/>
     </row>
@@ -1754,12 +1763,12 @@
   <sheetData>
     <row r="1" spans="1:2" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1772,7 +1781,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" s="5" t="str">
         <f>IF(owner &lt;&gt; "", owner, "")</f>
@@ -1872,17 +1881,17 @@
   <sheetData>
     <row r="1" spans="1:5" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="5" t="s">
@@ -1895,7 +1904,7 @@
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="5" t="s">
-        <v>6</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -1904,28 +1913,28 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="5"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="5"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="5"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="5"/>
@@ -1935,10 +1944,10 @@
       <c r="B11" s="7"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" s="30"/>
+      <c r="A12" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="35"/>
       <c r="C12" s="5"/>
       <c r="E12" s="6"/>
     </row>
@@ -1948,7 +1957,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="5"/>
@@ -1956,7 +1965,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="5"/>
@@ -1964,7 +1973,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="5"/>
@@ -1982,21 +1991,21 @@
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="7"/>
       <c r="B19" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C19" s="5"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="7"/>
       <c r="B20" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C20" s="5"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="7"/>
       <c r="B21" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C21" s="5"/>
     </row>
@@ -2006,7 +2015,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="5"/>
@@ -2059,89 +2068,89 @@
   <sheetData>
     <row r="1" spans="1:38" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
+        <v>8</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
     </row>
     <row r="6" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
+        <v>18</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="36"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
     </row>
     <row r="7" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="31"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="31"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
     </row>
     <row r="8" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="34"/>
+        <v>9</v>
+      </c>
+      <c r="B8" s="37"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="39"/>
     </row>
     <row r="9" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="32"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="34"/>
+        <v>52</v>
+      </c>
+      <c r="B9" s="37"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="39"/>
     </row>
     <row r="10" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="34"/>
+        <v>53</v>
+      </c>
+      <c r="B10" s="37"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="39"/>
     </row>
     <row r="11" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="31"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="31"/>
+        <v>12</v>
+      </c>
+      <c r="B11" s="36"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
     </row>
     <row r="12" spans="1:38" x14ac:dyDescent="0.2">
       <c r="W12" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="X12" s="20"/>
       <c r="Y12" s="20"/>
@@ -2163,16 +2172,16 @@
         <v>0</v>
       </c>
       <c r="B13" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="11" t="s">
         <v>10</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>11</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>3</v>
@@ -2181,97 +2190,97 @@
         <v>2</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I13" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="J13" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J13" s="10" t="s">
+      <c r="K13" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="K13" s="10" t="s">
+      <c r="L13" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="L13" s="10" t="s">
-        <v>15</v>
-      </c>
       <c r="M13" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N13" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="O13" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="O13" s="10" t="s">
+      <c r="P13" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q13" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="P13" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q13" s="10" t="s">
+      <c r="R13" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="R13" s="10" t="s">
+      <c r="S13" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="S13" s="10" t="s">
+      <c r="T13" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="T13" s="10" t="s">
+      <c r="U13" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="U13" s="10" t="s">
+      <c r="V13" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="V13" s="10" t="s">
+      <c r="W13" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="W13" s="10" t="s">
-        <v>78</v>
-      </c>
       <c r="X13" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y13" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="Y13" s="10" t="s">
+      <c r="Z13" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="Z13" s="10" t="s">
+      <c r="AA13" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="AB13" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="AC13" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="AD13" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="AE13" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="AA13" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="AB13" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC13" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="AD13" s="10" t="s">
+      <c r="AF13" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="AG13" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="AE13" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="AF13" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="AG13" s="10" t="s">
+      <c r="AH13" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="AI13" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="AH13" s="10" t="s">
+      <c r="AJ13" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="AK13" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="AI13" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="AJ13" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="AK13" s="10" t="s">
-        <v>89</v>
-      </c>
       <c r="AL13" s="10" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:38" x14ac:dyDescent="0.2">
@@ -3758,77 +3767,77 @@
   <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.5" style="36" customWidth="1"/>
-    <col min="2" max="2" width="22" style="36" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" style="36" customWidth="1"/>
-    <col min="4" max="4" width="32.6640625" style="36" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" style="36" customWidth="1"/>
-    <col min="6" max="6" width="28.33203125" style="36" customWidth="1"/>
-    <col min="7" max="7" width="19" style="36" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16" style="36" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" style="36" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.5" style="36" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5" style="36" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.83203125" style="36" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.83203125" style="36" customWidth="1"/>
-    <col min="14" max="16384" width="8.83203125" style="36"/>
+    <col min="1" max="1" width="17.5" style="30" customWidth="1"/>
+    <col min="2" max="2" width="22" style="30" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="30" customWidth="1"/>
+    <col min="4" max="4" width="32.6640625" style="30" customWidth="1"/>
+    <col min="5" max="5" width="18.33203125" style="30" customWidth="1"/>
+    <col min="6" max="6" width="28.33203125" style="30" customWidth="1"/>
+    <col min="7" max="7" width="19" style="30" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16" style="30" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" style="30" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.5" style="30" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5" style="30" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.83203125" style="30" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.83203125" style="30" customWidth="1"/>
+    <col min="14" max="16384" width="8.83203125" style="30"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.2">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="B1" s="29"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" s="31"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="31"/>
+      <c r="B3" s="31"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>155</v>
+      </c>
+      <c r="F4" s="33" t="s">
+        <v>153</v>
+      </c>
+      <c r="G4" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="H4" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="I4" s="33" t="s">
+        <v>154</v>
+      </c>
+      <c r="J4" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="35"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="37" t="s">
-        <v>153</v>
-      </c>
-      <c r="B2" s="37"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="37"/>
-      <c r="B3" s="37"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="38" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="38" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="39" t="s">
-        <v>90</v>
-      </c>
-      <c r="D4" s="39" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="39" t="s">
-        <v>159</v>
-      </c>
-      <c r="F4" s="39" t="s">
+      <c r="K4" s="33" t="s">
+        <v>156</v>
+      </c>
+      <c r="L4" s="33" t="s">
         <v>157</v>
       </c>
-      <c r="G4" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="H4" s="39" t="s">
-        <v>155</v>
-      </c>
-      <c r="I4" s="39" t="s">
+      <c r="M4" s="33" t="s">
         <v>158</v>
-      </c>
-      <c r="J4" s="39" t="s">
-        <v>156</v>
-      </c>
-      <c r="K4" s="39" t="s">
-        <v>160</v>
-      </c>
-      <c r="L4" s="39" t="s">
-        <v>161</v>
-      </c>
-      <c r="M4" s="39" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -4137,32 +4146,32 @@
   <sheetData>
     <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>57</v>
-      </c>
       <c r="F4" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -4322,35 +4331,35 @@
   <sheetData>
     <row r="1" spans="1:7" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="10" t="s">
         <v>67</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -4529,29 +4538,29 @@
   <sheetData>
     <row r="1" spans="1:5" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="10" t="s">
         <v>99</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -4696,12 +4705,12 @@
   <sheetData>
     <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -4709,7 +4718,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B4" s="26"/>
     </row>
@@ -4721,16 +4730,16 @@
         <v>1</v>
       </c>
       <c r="C6" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="E6" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="F6" s="10" t="s">
         <v>106</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -4880,7 +4889,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{246082EA-DAAB-1649-871C-B98419509DC8}">
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.1640625" style="2" customWidth="1"/>
@@ -4894,19 +4903,19 @@
   <sheetData>
     <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B2" s="4"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="5"/>
@@ -4916,7 +4925,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="5"/>
@@ -4940,7 +4949,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="5"/>
@@ -4950,13 +4959,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="7"/>
       <c r="B12" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -4966,7 +4975,7 @@
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="7"/>
       <c r="B13" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
@@ -4976,7 +4985,7 @@
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="7"/>
       <c r="B14" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
@@ -4988,13 +4997,13 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="7"/>
       <c r="B17" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -5004,7 +5013,7 @@
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="7"/>
       <c r="B18" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -5016,13 +5025,13 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="7"/>
       <c r="B21" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
@@ -5032,7 +5041,7 @@
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="7"/>
       <c r="B22" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
@@ -5042,7 +5051,7 @@
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="7"/>
       <c r="B23" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -5054,13 +5063,13 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="7"/>
       <c r="B26" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
@@ -5070,7 +5079,7 @@
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="7"/>
       <c r="B27" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -5080,7 +5089,7 @@
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="7"/>
       <c r="B28" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
@@ -5090,7 +5099,7 @@
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="7"/>
       <c r="B29" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
@@ -5102,13 +5111,13 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="7"/>
       <c r="B32" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
@@ -5118,7 +5127,7 @@
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="7"/>
       <c r="B33" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
@@ -5130,13 +5139,13 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="7"/>
       <c r="B36" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
@@ -5146,7 +5155,7 @@
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="7"/>
       <c r="B37" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="5"/>
@@ -5156,7 +5165,7 @@
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="7"/>
       <c r="B38" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>
@@ -5166,7 +5175,7 @@
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="7"/>
       <c r="B39" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
@@ -5178,13 +5187,13 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="7"/>
       <c r="B42" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
@@ -5194,7 +5203,7 @@
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="7"/>
       <c r="B43" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
@@ -5204,7 +5213,7 @@
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="7"/>
       <c r="B44" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5"/>
@@ -5214,7 +5223,7 @@
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="7"/>
       <c r="B45" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
@@ -5226,13 +5235,13 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="7"/>
       <c r="B48" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5"/>
@@ -5242,7 +5251,7 @@
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="7"/>
       <c r="B49" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="5"/>
@@ -5252,7 +5261,7 @@
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="7"/>
       <c r="B50" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
@@ -5262,7 +5271,7 @@
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="7"/>
       <c r="B51" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C51" s="5"/>
       <c r="D51" s="5"/>
@@ -5272,7 +5281,7 @@
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="7"/>
       <c r="B52" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
@@ -5282,7 +5291,7 @@
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="7"/>
       <c r="B53" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5"/>
@@ -5294,13 +5303,13 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="7"/>
       <c r="B56" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5"/>
@@ -5310,7 +5319,7 @@
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="7"/>
       <c r="B57" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5"/>
@@ -5320,7 +5329,7 @@
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="7"/>
       <c r="B58" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
@@ -5330,7 +5339,7 @@
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="7"/>
       <c r="B59" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C59" s="5"/>
       <c r="D59" s="5"/>
@@ -5342,13 +5351,13 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
-        <v>134</v>
+        <v>163</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="7"/>
       <c r="B62" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C62" s="5"/>
       <c r="D62" s="5"/>
@@ -5358,7 +5367,7 @@
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="7"/>
       <c r="B63" s="2" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="C63" s="5"/>
       <c r="D63" s="5"/>
@@ -5368,7 +5377,7 @@
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="7"/>
       <c r="B64" s="2" t="s">
-        <v>114</v>
+        <v>164</v>
       </c>
       <c r="C64" s="5"/>
       <c r="D64" s="5"/>
@@ -5377,28 +5386,16 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="7"/>
-      <c r="B65" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C65" s="5"/>
-      <c r="D65" s="5"/>
-      <c r="E65" s="5"/>
-      <c r="F65" s="5"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A66" s="7"/>
-      <c r="B66" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="C66" s="5"/>
-      <c r="D66" s="5"/>
-      <c r="E66" s="5"/>
-      <c r="F66" s="5"/>
+      <c r="A66" s="7" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="7"/>
       <c r="B67" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C67" s="5"/>
       <c r="D67" s="5"/>
@@ -5408,7 +5405,7 @@
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="7"/>
       <c r="B68" s="2" t="s">
-        <v>82</v>
+        <v>112</v>
       </c>
       <c r="C68" s="5"/>
       <c r="D68" s="5"/>
@@ -5418,7 +5415,7 @@
     <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="7"/>
       <c r="B69" s="2" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C69" s="5"/>
       <c r="D69" s="5"/>
@@ -5428,7 +5425,7 @@
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="7"/>
       <c r="B70" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C70" s="5"/>
       <c r="D70" s="5"/>
@@ -5438,7 +5435,7 @@
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="7"/>
       <c r="B71" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C71" s="5"/>
       <c r="D71" s="5"/>
@@ -5448,7 +5445,7 @@
     <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="7"/>
       <c r="B72" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
@@ -5458,7 +5455,7 @@
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="7"/>
       <c r="B73" s="2" t="s">
-        <v>122</v>
+        <v>81</v>
       </c>
       <c r="C73" s="5"/>
       <c r="D73" s="5"/>
@@ -5468,7 +5465,7 @@
     <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="7"/>
       <c r="B74" s="2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C74" s="5"/>
       <c r="D74" s="5"/>
@@ -5478,7 +5475,7 @@
     <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="7"/>
       <c r="B75" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" s="5"/>
@@ -5488,7 +5485,7 @@
     <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="7"/>
       <c r="B76" s="2" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="C76" s="5"/>
       <c r="D76" s="5"/>
@@ -5498,7 +5495,7 @@
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="7"/>
       <c r="B77" s="2" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="C77" s="5"/>
       <c r="D77" s="5"/>
@@ -5508,7 +5505,7 @@
     <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="7"/>
       <c r="B78" s="2" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="C78" s="5"/>
       <c r="D78" s="5"/>
@@ -5518,7 +5515,7 @@
     <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="7"/>
       <c r="B79" s="2" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="C79" s="5"/>
       <c r="D79" s="5"/>
@@ -5528,16 +5525,66 @@
     <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="7"/>
       <c r="B80" s="2" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="C80" s="5"/>
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
       <c r="F80" s="5"/>
     </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A81" s="7"/>
+      <c r="B81" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C81" s="5"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A82" s="7"/>
+      <c r="B82" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C82" s="5"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A83" s="7"/>
+      <c r="B83" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C83" s="5"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A84" s="7"/>
+      <c r="B84" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C84" s="5"/>
+      <c r="D84" s="5"/>
+      <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A85" s="7"/>
+      <c r="B85" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C85" s="5"/>
+      <c r="D85" s="5"/>
+      <c r="E85" s="5"/>
+      <c r="F85" s="5"/>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="1" sqref="G4:AE43 C4:F7 C9:F45 C48:F53 C56:F59 C62:F80" xr:uid="{AEB39A8F-9810-ED4E-9F27-465756D4623D}"/>
+    <dataValidation allowBlank="1" sqref="G4:AE43 C4:F7 C9:F45 C48:F53 C67:F85 C56:F59 C62:F64" xr:uid="{AEB39A8F-9810-ED4E-9F27-465756D4623D}"/>
     <dataValidation type="list" allowBlank="1" sqref="C8:F8" xr:uid="{DF709D8D-57D8-6842-9BBE-389F6303D2F1}">
       <formula1>"api,athena,azure,bigquery,clickhouse,databricks,db2,denodo,dremio,duckdb,glue,cloudsql,informix,kafka,kinesis,mysql,local,oracle,postgresql,presto,pubsub,redshift,s3,sftp,snowflake,sqlserver,synapse,trino,vertica,custom"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Add relationships to template
</commit_message>
<xml_diff>
--- a/odcs-template.xlsx
+++ b/odcs-template.xlsx
@@ -1,29 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jochen/Projects/open-data-contract-standard-excel-template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fb/IdeaProjects/entropy-data/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B8EC82A-F0B9-0B43-8073-AB65EEFA9D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1AEC928-3B3E-6A48-BC07-BADEA98D1A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="8" r:id="rId1"/>
     <sheet name="Fundamentals" sheetId="10" r:id="rId2"/>
     <sheet name="Schema &lt;table_name&gt;" sheetId="3" r:id="rId3"/>
-    <sheet name="Quality" sheetId="21" r:id="rId4"/>
-    <sheet name="Support" sheetId="12" r:id="rId5"/>
-    <sheet name="Team" sheetId="13" r:id="rId6"/>
-    <sheet name="Roles" sheetId="16" r:id="rId7"/>
-    <sheet name="SLA" sheetId="17" r:id="rId8"/>
-    <sheet name="Servers" sheetId="20" r:id="rId9"/>
-    <sheet name="Pricing" sheetId="15" r:id="rId10"/>
-    <sheet name="Custom Properties" sheetId="11" r:id="rId11"/>
+    <sheet name="Relationships" sheetId="23" r:id="rId4"/>
+    <sheet name="Quality" sheetId="21" r:id="rId5"/>
+    <sheet name="Support" sheetId="12" r:id="rId6"/>
+    <sheet name="Team" sheetId="13" r:id="rId7"/>
+    <sheet name="Roles" sheetId="16" r:id="rId8"/>
+    <sheet name="SLA" sheetId="17" r:id="rId9"/>
+    <sheet name="Servers" sheetId="20" r:id="rId10"/>
+    <sheet name="Pricing" sheetId="15" r:id="rId11"/>
+    <sheet name="Custom Properties" sheetId="11" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="apiVersion">Fundamentals!$C$5</definedName>
@@ -43,7 +44,8 @@
     <definedName name="price.priceCurrency">Pricing!$B$5</definedName>
     <definedName name="price.priceUnit">Pricing!$B$6</definedName>
     <definedName name="quality">Quality!$A$4:$AZ$300</definedName>
-    <definedName name="roles" localSheetId="6">Roles!$A$4:$E$1000</definedName>
+    <definedName name="relationships">Relationships!$A$4:$AZ$300</definedName>
+    <definedName name="roles" localSheetId="7">Roles!$A$4:$E$1000</definedName>
     <definedName name="schema.businessName" localSheetId="2">'Schema &lt;table_name&gt;'!$B$8</definedName>
     <definedName name="schema.dataGranularityDescription" localSheetId="2">'Schema &lt;table_name&gt;'!$B$10</definedName>
     <definedName name="schema.description" localSheetId="2">'Schema &lt;table_name&gt;'!$B$7</definedName>
@@ -111,7 +113,7 @@
     <definedName name="servers.sqlserver.schema">Servers!$C$59</definedName>
     <definedName name="servers.type">Servers!$C$8</definedName>
     <definedName name="slaDefaultElement">SLA!$B$4</definedName>
-    <definedName name="slaProperties" localSheetId="7">SLA!$A$6:$F$1002</definedName>
+    <definedName name="slaProperties" localSheetId="8">SLA!$A$6:$F$1002</definedName>
     <definedName name="status">Fundamentals!$C$10</definedName>
     <definedName name="support">Support!$A$4:$F$1000</definedName>
     <definedName name="tags">Fundamentals!$C$23</definedName>
@@ -137,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="172">
   <si>
     <t>Property</t>
   </si>
@@ -642,6 +644,24 @@
   </si>
   <si>
     <t>v3.0.2</t>
+  </si>
+  <si>
+    <t>Relationships</t>
+  </si>
+  <si>
+    <t>Define relationships between schemas by mapping properties from one schema to another (e.g., foreign keys).</t>
+  </si>
+  <si>
+    <t>Use schema.property dot syntax (e.g., orders.customer_id). Comma-separated for composite keys. Level: 'schema' or 'property'.</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>From</t>
+  </si>
+  <si>
+    <t>To</t>
   </si>
 </sst>
 </file>
@@ -968,7 +988,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1343,6 +1370,26 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{2169EE2B-12FA-C14F-81DC-D91B65338178}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:I31"/>
@@ -1703,6 +1750,712 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{246082EA-DAAB-1649-871C-B98419509DC8}">
+  <dimension ref="A1:F85"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.1640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="33.1640625" style="2" customWidth="1"/>
+    <col min="3" max="6" width="36.1640625" style="2" customWidth="1"/>
+    <col min="7" max="22" width="15" style="2" customWidth="1"/>
+    <col min="23" max="30" width="32.83203125" style="2" customWidth="1"/>
+    <col min="31" max="31" width="34.6640625" style="2" customWidth="1"/>
+    <col min="32" max="16384" width="8.83203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B2" s="4"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="7"/>
+      <c r="B12" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="7"/>
+      <c r="B13" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="7"/>
+      <c r="B14" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="7"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="7"/>
+      <c r="B17" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="7"/>
+      <c r="B18" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" s="7" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="7"/>
+      <c r="B21" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="7"/>
+      <c r="B22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="7"/>
+      <c r="B23" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="7"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" s="7" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="7"/>
+      <c r="B26" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" s="7"/>
+      <c r="B27" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="7"/>
+      <c r="B28" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="7"/>
+      <c r="B29" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" s="7"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" s="7" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" s="7"/>
+      <c r="B32" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33" s="7"/>
+      <c r="B33" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" s="7"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" s="7"/>
+      <c r="B36" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" s="7"/>
+      <c r="B37" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" s="7"/>
+      <c r="B38" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39" s="7"/>
+      <c r="B39" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A40" s="7"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41" s="7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42" s="7"/>
+      <c r="B42" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A43" s="7"/>
+      <c r="B43" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C43" s="5"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44" s="7"/>
+      <c r="B44" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45" s="7"/>
+      <c r="B45" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46" s="7"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" s="7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48" s="7"/>
+      <c r="B48" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A49" s="7"/>
+      <c r="B49" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A50" s="7"/>
+      <c r="B50" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C50" s="5"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A51" s="7"/>
+      <c r="B51" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A52" s="7"/>
+      <c r="B52" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C52" s="5"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A53" s="7"/>
+      <c r="B53" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A54" s="7"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A55" s="7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A56" s="7"/>
+      <c r="B56" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A57" s="7"/>
+      <c r="B57" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A58" s="7"/>
+      <c r="B58" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A59" s="7"/>
+      <c r="B59" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A60" s="7"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A61" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A62" s="7"/>
+      <c r="B62" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C62" s="5"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A63" s="7"/>
+      <c r="B63" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C63" s="5"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A64" s="7"/>
+      <c r="B64" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C64" s="5"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A65" s="7"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A66" s="7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A67" s="7"/>
+      <c r="B67" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C67" s="5"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A68" s="7"/>
+      <c r="B68" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C68" s="5"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A69" s="7"/>
+      <c r="B69" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A70" s="7"/>
+      <c r="B70" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C70" s="5"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A71" s="7"/>
+      <c r="B71" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C71" s="5"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A72" s="7"/>
+      <c r="B72" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A73" s="7"/>
+      <c r="B73" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C73" s="5"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="5"/>
+      <c r="F73" s="5"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A74" s="7"/>
+      <c r="B74" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C74" s="5"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="5"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A75" s="7"/>
+      <c r="B75" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C75" s="5"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="5"/>
+      <c r="F75" s="5"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A76" s="7"/>
+      <c r="B76" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C76" s="5"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A77" s="7"/>
+      <c r="B77" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C77" s="5"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A78" s="7"/>
+      <c r="B78" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C78" s="5"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A79" s="7"/>
+      <c r="B79" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C79" s="5"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="5"/>
+      <c r="F79" s="5"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A80" s="7"/>
+      <c r="B80" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C80" s="5"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A81" s="7"/>
+      <c r="B81" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C81" s="5"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A82" s="7"/>
+      <c r="B82" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C82" s="5"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A83" s="7"/>
+      <c r="B83" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C83" s="5"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A84" s="7"/>
+      <c r="B84" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C84" s="5"/>
+      <c r="D84" s="5"/>
+      <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A85" s="7"/>
+      <c r="B85" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C85" s="5"/>
+      <c r="D85" s="5"/>
+      <c r="E85" s="5"/>
+      <c r="F85" s="5"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation allowBlank="1" sqref="G4:AE43 C4:F7 C9:F45 C48:F53 C67:F85 C56:F59 C62:F64" xr:uid="{AEB39A8F-9810-ED4E-9F27-465756D4623D}"/>
+    <dataValidation type="list" allowBlank="1" sqref="C8:F8" xr:uid="{DF709D8D-57D8-6842-9BBE-389F6303D2F1}">
+      <formula1>"api,athena,azure,bigquery,clickhouse,databricks,db2,denodo,dremio,duckdb,glue,cloudsql,informix,kafka,kinesis,mysql,local,oracle,postgresql,presto,pubsub,redshift,s3,sftp,snowflake,sqlserver,synapse,trino,vertica,custom"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C95CB51A-C5C4-224E-AA94-69EA1F503FF6}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1751,7 +2504,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29635FC6-19E5-6E43-84D3-3161FAC792B3}">
   <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3763,6 +4516,198 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0C8C2B4-64D3-DB4C-BBDA-0F192B30B9A9}">
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="8.33203125" style="30" customWidth="1"/>
+    <col min="2" max="2" width="13" style="30" customWidth="1"/>
+    <col min="3" max="3" width="48.5" style="30" customWidth="1"/>
+    <col min="4" max="4" width="42.83203125" style="30" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" style="30" customWidth="1"/>
+    <col min="6" max="16384" width="8.83203125" style="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="24" x14ac:dyDescent="0.2">
+      <c r="A1" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="29"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="31" t="s">
+        <v>167</v>
+      </c>
+      <c r="B2" s="31"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="31" t="s">
+        <v>168</v>
+      </c>
+      <c r="B3" s="31"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="32" t="s">
+        <v>169</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>170</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E5:E21">
+    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
+      <formula>C5="sql"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="8">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Description" prompt="A human-readable description of the relationship. Explain the business context or purpose of how the source and target are related." sqref="E4" xr:uid="{EE4A1054-F15A-664C-B875-762503081248}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Type" prompt="Type of the relationship column(s)." sqref="B4" xr:uid="{41A27CD9-820D-2E48-B8C9-300C785AF670}"/>
+    <dataValidation allowBlank="1" showErrorMessage="1" sqref="A4" xr:uid="{C01DBA5A-CD2D-5340-88E8-907CC68A70F7}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="From" prompt="Source property or schema of the relationship. Use schema.property dot notation (e.g., orders.customer_id). For composite keys at schema level, use comma-separated values (e.g., orders.order_id, orders.line_id)." sqref="C4" xr:uid="{BF1567BA-BD98-8A43-A618-6A6EA6B0FD4E}"/>
+    <dataValidation allowBlank="1" sqref="C22:E42" xr:uid="{8EB79343-A157-4243-B7EE-3C19030C4E99}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Level" prompt="Select if the relationship shall be defined on schema or property level. Use schema level for composite keys." sqref="A5:A100" xr:uid="{64056970-A677-8843-8D33-4CF3120F6E95}">
+      <formula1>"schema,property"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Type" prompt="Type of the relationship column(s)." sqref="B5:B100" xr:uid="{F3BC2467-11B9-1846-9D62-3055019048A0}">
+      <formula1>"foreignKey,references,mapsTo"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="To" prompt="Target property or schema the source maps to. Use schema.property dot notation (e.g., customers.id). For composite keys at schema level, use comma-separated values matching the order of the 'From' fields." sqref="D4" xr:uid="{7117A4CC-D0A3-894D-B5D8-FA6426CA462E}"/>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC0F4C5A-BE41-6140-9B9B-80B8DB7D1AD7}">
   <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4130,10 +5075,11 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Rule" prompt="The predefined data quality rule from the library._x000a_Only appliable if &quot;Quality Type&quot; is set to &quot;library&quot; or empty (which is library by default, if a rule is defined)" sqref="E4" xr:uid="{4E8AA24F-1E70-FF4C-81CC-D9A25B05246C}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90FB3633-F435-1B44-A99B-F400ACF77C57}">
   <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4318,7 +5264,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD55E6DF-E5C5-C142-BA93-791862A30BE7}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4523,7 +5469,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B433535-9968-AF4C-822D-F1478F01E2E0}">
   <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4690,7 +5636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09C18618-CA09-244F-9E12-D5D128AED5CE}">
   <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4885,710 +5831,4 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{246082EA-DAAB-1649-871C-B98419509DC8}">
-  <dimension ref="A1:F85"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="6.1640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="33.1640625" style="2" customWidth="1"/>
-    <col min="3" max="6" width="36.1640625" style="2" customWidth="1"/>
-    <col min="7" max="22" width="15" style="2" customWidth="1"/>
-    <col min="23" max="30" width="32.83203125" style="2" customWidth="1"/>
-    <col min="31" max="31" width="34.6640625" style="2" customWidth="1"/>
-    <col min="32" max="16384" width="8.83203125" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="4"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="7"/>
-      <c r="B12" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="7"/>
-      <c r="B13" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="7"/>
-      <c r="B14" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="7"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="7" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="7"/>
-      <c r="B17" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="7"/>
-      <c r="B18" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="7"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="7"/>
-      <c r="B21" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="7"/>
-      <c r="B22" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="7"/>
-      <c r="B23" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="7"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="7" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="7"/>
-      <c r="B26" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="7"/>
-      <c r="B27" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="7"/>
-      <c r="B28" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="7"/>
-      <c r="B29" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="7"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31" s="7" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" s="7"/>
-      <c r="B32" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A33" s="7"/>
-      <c r="B33" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="7"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="7" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="7"/>
-      <c r="B36" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A37" s="7"/>
-      <c r="B37" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A38" s="7"/>
-      <c r="B38" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A39" s="7"/>
-      <c r="B39" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A40" s="7"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A41" s="7" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A42" s="7"/>
-      <c r="B42" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A43" s="7"/>
-      <c r="B43" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="C43" s="5"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="5"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A44" s="7"/>
-      <c r="B44" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A45" s="7"/>
-      <c r="B45" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A46" s="7"/>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A47" s="7" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A48" s="7"/>
-      <c r="B48" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A49" s="7"/>
-      <c r="B49" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A50" s="7"/>
-      <c r="B50" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C50" s="5"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5"/>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A51" s="7"/>
-      <c r="B51" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A52" s="7"/>
-      <c r="B52" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5"/>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A53" s="7"/>
-      <c r="B53" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5"/>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A54" s="7"/>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A55" s="7" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A56" s="7"/>
-      <c r="B56" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A57" s="7"/>
-      <c r="B57" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C57" s="5"/>
-      <c r="D57" s="5"/>
-      <c r="E57" s="5"/>
-      <c r="F57" s="5"/>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A58" s="7"/>
-      <c r="B58" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A59" s="7"/>
-      <c r="B59" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="5"/>
-      <c r="F59" s="5"/>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A60" s="7"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A61" s="7" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A62" s="7"/>
-      <c r="B62" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A63" s="7"/>
-      <c r="B63" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A64" s="7"/>
-      <c r="B64" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
-      <c r="F64" s="5"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A65" s="7"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A66" s="7" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A67" s="7"/>
-      <c r="B67" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-      <c r="F67" s="5"/>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A68" s="7"/>
-      <c r="B68" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5"/>
-      <c r="E68" s="5"/>
-      <c r="F68" s="5"/>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A69" s="7"/>
-      <c r="B69" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A70" s="7"/>
-      <c r="B70" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C70" s="5"/>
-      <c r="D70" s="5"/>
-      <c r="E70" s="5"/>
-      <c r="F70" s="5"/>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A71" s="7"/>
-      <c r="B71" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C71" s="5"/>
-      <c r="D71" s="5"/>
-      <c r="E71" s="5"/>
-      <c r="F71" s="5"/>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A72" s="7"/>
-      <c r="B72" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5"/>
-      <c r="E72" s="5"/>
-      <c r="F72" s="5"/>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A73" s="7"/>
-      <c r="B73" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C73" s="5"/>
-      <c r="D73" s="5"/>
-      <c r="E73" s="5"/>
-      <c r="F73" s="5"/>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A74" s="7"/>
-      <c r="B74" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C74" s="5"/>
-      <c r="D74" s="5"/>
-      <c r="E74" s="5"/>
-      <c r="F74" s="5"/>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A75" s="7"/>
-      <c r="B75" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C75" s="5"/>
-      <c r="D75" s="5"/>
-      <c r="E75" s="5"/>
-      <c r="F75" s="5"/>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A76" s="7"/>
-      <c r="B76" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5"/>
-      <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A77" s="7"/>
-      <c r="B77" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C77" s="5"/>
-      <c r="D77" s="5"/>
-      <c r="E77" s="5"/>
-      <c r="F77" s="5"/>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A78" s="7"/>
-      <c r="B78" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C78" s="5"/>
-      <c r="D78" s="5"/>
-      <c r="E78" s="5"/>
-      <c r="F78" s="5"/>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A79" s="7"/>
-      <c r="B79" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="C79" s="5"/>
-      <c r="D79" s="5"/>
-      <c r="E79" s="5"/>
-      <c r="F79" s="5"/>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A80" s="7"/>
-      <c r="B80" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C80" s="5"/>
-      <c r="D80" s="5"/>
-      <c r="E80" s="5"/>
-      <c r="F80" s="5"/>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A81" s="7"/>
-      <c r="B81" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C81" s="5"/>
-      <c r="D81" s="5"/>
-      <c r="E81" s="5"/>
-      <c r="F81" s="5"/>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A82" s="7"/>
-      <c r="B82" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C82" s="5"/>
-      <c r="D82" s="5"/>
-      <c r="E82" s="5"/>
-      <c r="F82" s="5"/>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A83" s="7"/>
-      <c r="B83" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C83" s="5"/>
-      <c r="D83" s="5"/>
-      <c r="E83" s="5"/>
-      <c r="F83" s="5"/>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A84" s="7"/>
-      <c r="B84" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C84" s="5"/>
-      <c r="D84" s="5"/>
-      <c r="E84" s="5"/>
-      <c r="F84" s="5"/>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A85" s="7"/>
-      <c r="B85" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C85" s="5"/>
-      <c r="D85" s="5"/>
-      <c r="E85" s="5"/>
-      <c r="F85" s="5"/>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="1" sqref="G4:AE43 C4:F7 C9:F45 C48:F53 C67:F85 C56:F59 C62:F64" xr:uid="{AEB39A8F-9810-ED4E-9F27-465756D4623D}"/>
-    <dataValidation type="list" allowBlank="1" sqref="C8:F8" xr:uid="{DF709D8D-57D8-6842-9BBE-389F6303D2F1}">
-      <formula1>"api,athena,azure,bigquery,clickhouse,databricks,db2,denodo,dremio,duckdb,glue,cloudsql,informix,kafka,kinesis,mysql,local,oracle,postgresql,presto,pubsub,redshift,s3,sftp,snowflake,sqlserver,synapse,trino,vertica,custom"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
copy over from v3.2.0
</commit_message>
<xml_diff>
--- a/odcs-template.xlsx
+++ b/odcs-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakob/entropyData/open-data-contract-standard-excel-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1031AD6A-ED8F-9542-9505-273B1DC3029A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{342FE4F4-9DE3-3540-BE91-7790BCC57F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
     <definedName name="price.priceUnit">Pricing!$B$6</definedName>
     <definedName name="quality">Quality!$A$4:$BF$300</definedName>
     <definedName name="relationships">Relationships!$A$4:$AZ$300</definedName>
-    <definedName name="roles" localSheetId="7">Roles!$C$4:$BB$1000</definedName>
+    <definedName name="roles" localSheetId="7">Roles!$A$4:$AZ$1000</definedName>
     <definedName name="schema.businessName" localSheetId="2">'Schema &lt;table_name&gt;'!$B$8</definedName>
     <definedName name="schema.context.instructions" localSheetId="2">'Schema &lt;table_name&gt;'!$B$13</definedName>
     <definedName name="schema.dataGranularityDescription" localSheetId="2">'Schema &lt;table_name&gt;'!$B$10</definedName>
@@ -1124,7 +1124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1227,7 +1227,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -18980,7 +18979,7 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="4" t="s">
         <v>248</v>
       </c>
     </row>

</xml_diff>